<commit_message>
CI ready clean framework setup
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/planetrehab-testdata.xlsx
+++ b/src/main/resources/testdata/planetrehab-testdata.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Selenium Workspace\planetrehab-automation-framework\src\main\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D82281-7445-4008-B878-215E37EDB4EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F343A7A8-769B-4959-9B7B-34D0B3C0A00B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="RegisterPatient" sheetId="2" r:id="rId2"/>
+    <sheet name="CareProfileCreation" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -40,12 +41,6 @@
     <t>validLogin</t>
   </si>
   <si>
-    <t>Youngsoft@12345</t>
-  </si>
-  <si>
-    <t>eliteptadmin@yopmail.com</t>
-  </si>
-  <si>
     <t>firstName</t>
   </si>
   <si>
@@ -86,6 +81,12 @@
   </si>
   <si>
     <t>NO</t>
+  </si>
+  <si>
+    <t>pudar.r@youngsoft.in</t>
+  </si>
+  <si>
+    <t>Pass@12345</t>
   </si>
 </sst>
 </file>
@@ -456,14 +457,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="2" width="18.21875" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="1" max="1" width="14.81640625" customWidth="1"/>
+    <col min="2" max="2" width="22.1796875" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -482,15 +483,15 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -513,67 +514,76 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38E2E230-E218-44EA-B71E-ACA7B3F05880}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="12.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>9</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>11</v>
       </c>
       <c r="C2" s="7">
         <v>35588</v>
       </c>
       <c r="D2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>12</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>14</v>
       </c>
       <c r="C3" s="7">
         <v>32874</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DC486E4-E031-42DE-9020-2A211231CB75}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>